<commit_message>
🎯 Strike: IDN URLs as Corsearch stores them; p6 halves to find the existing account
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brand-protection/2026-09-28/strike/01-mono_other-p8.xlsx
+++ b/brand-protection/2026-09-28/strike/01-mono_other-p8.xlsx
@@ -4322,7 +4322,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>https://xn----7sbajchefi3c5abkjc2d4i.xn--p1ai/</t>
+          <t>https://фаергард-поволжье.рф/</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4344,7 +4344,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>https://xn----7sblece8bdveh9l.xn--p1ai/</t>
+          <t>https://дренаж-пермь.рф/</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4366,7 +4366,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>https://xn----7sbqgez1bcecc.xn--p1ai/</t>
+          <t>https://аутизм-тест.рф/</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4388,7 +4388,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>https://xn----8sba7blnqd3a.xn--p1ai/</t>
+          <t>https://рц-атлант.рф/</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4410,7 +4410,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>https://xn----ctbbmvm0c3a2c.xn--p1ai/</t>
+          <t>https://кмв-цветы.рф/</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4432,7 +4432,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>https://xn----dtbfea6a0akik4e6a9a.xn--p1ai/</t>
+          <t>https://люстры-дешево.рф/</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4454,7 +4454,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>https://xn--80aaah0dhi.xn--p1ai/</t>
+          <t>https://параван.рф/</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4476,7 +4476,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>https://xn--80aabbgg8aaod1ahg0k3e.xn--p1ai/</t>
+          <t>https://банябочкавикинг.рф/</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4498,7 +4498,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>https://xn--80abcf9dqr.xn--p1ai/</t>
+          <t>https://вбуграх.рф/</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4520,7 +4520,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>https://xn--80ahbnxidcjb.xn--p1ai/</t>
+          <t>https://природадом.рф/</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4542,7 +4542,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>https://xn--80ahklijc.xn--p1ai/</t>
+          <t>https://домакзн.рф/</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -4564,7 +4564,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>https://xn--90ahpcrbldgh1j.xn--p1ai/</t>
+          <t>https://электросбор.рф/</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4586,7 +4586,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>https://xn--90aitipgc.net/</t>
+          <t>https://мостбет.net/</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4608,7 +4608,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>https://xn--90aitipgc.su/</t>
+          <t>https://мостбет.su/</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">

</xml_diff>